<commit_message>
adding table-nested, uploader and pdf-viewer
</commit_message>
<xml_diff>
--- a/database/excels/organization/base-seeder.xlsx
+++ b/database/excels/organization/base-seeder.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/monoland/Platform/monoland/database/excels/organization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B79BF79C-9FC1-9C4B-BFF6-A425A59C9FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{406F0947-9BC9-294B-9128-3304260F2C65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="500" windowWidth="33580" windowHeight="20500" activeTab="2" xr2:uid="{94E1010F-4E68-D749-BBCF-3803F804C4FE}"/>
+    <workbookView xWindow="20" yWindow="500" windowWidth="33580" windowHeight="20500" activeTab="1" xr2:uid="{94E1010F-4E68-D749-BBCF-3803F804C4FE}"/>
   </bookViews>
   <sheets>
     <sheet name="module" sheetId="2" r:id="rId1"/>
@@ -218,9 +218,6 @@
     <t>Jenis Jabatan</t>
   </si>
   <si>
-    <t>Jenis Peta Jabatan</t>
-  </si>
-  <si>
     <t>Peta Fungsional</t>
   </si>
   <si>
@@ -387,6 +384,9 @@
   </si>
   <si>
     <t>workunitread/:workunitread/formation</t>
+  </si>
+  <si>
+    <t>Tingkat Jabatan</t>
   </si>
 </sst>
 </file>
@@ -906,16 +906,16 @@
         <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F3" t="s">
         <v>28</v>
       </c>
       <c r="G3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H3" s="4" t="b">
         <v>0</v>
@@ -929,22 +929,22 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F4" t="s">
         <v>28</v>
       </c>
       <c r="G4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H4" s="4" t="b">
         <v>0</v>
@@ -953,7 +953,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -967,16 +967,16 @@
         <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F5" t="s">
         <v>28</v>
       </c>
       <c r="G5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H5" s="4" t="b">
         <v>0</v>
@@ -990,22 +990,22 @@
         <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F6" t="s">
         <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H6" s="4" t="b">
         <v>0</v>
@@ -1019,22 +1019,22 @@
         <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F7" t="s">
         <v>28</v>
       </c>
       <c r="G7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H7" s="4" t="b">
         <v>0</v>
@@ -1043,7 +1043,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -1051,22 +1051,22 @@
         <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F8" t="s">
         <v>28</v>
       </c>
       <c r="G8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H8" s="4" t="b">
         <v>0</v>
@@ -1080,22 +1080,22 @@
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F9" t="s">
         <v>28</v>
       </c>
       <c r="G9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H9" s="4" t="b">
         <v>0</v>
@@ -1104,7 +1104,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -1121,13 +1121,13 @@
         <v>43</v>
       </c>
       <c r="E10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F10" t="s">
         <v>28</v>
       </c>
       <c r="G10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H10" s="4" t="b">
         <v>0</v>
@@ -1136,7 +1136,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
@@ -1150,16 +1150,16 @@
         <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F11" t="s">
         <v>28</v>
       </c>
       <c r="G11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H11" s="4" t="b">
         <v>0</v>
@@ -1182,7 +1182,7 @@
         <v>42</v>
       </c>
       <c r="E12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F12" t="s">
         <v>28</v>
@@ -1202,22 +1202,22 @@
         <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F13" t="s">
         <v>28</v>
       </c>
       <c r="G13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H13" s="4" t="b">
         <v>0</v>
@@ -1231,22 +1231,22 @@
         <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F14" t="s">
         <v>28</v>
       </c>
       <c r="G14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H14" s="4" t="b">
         <v>0</v>
@@ -1255,7 +1255,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
@@ -1292,22 +1292,22 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16" t="s">
         <v>81</v>
       </c>
-      <c r="C16" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" t="s">
-        <v>82</v>
-      </c>
       <c r="E16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F16" t="s">
         <v>28</v>
       </c>
       <c r="G16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H16" s="4" t="b">
         <v>0</v>
@@ -1321,22 +1321,22 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D17" t="s">
         <v>45</v>
       </c>
       <c r="E17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F17" t="s">
         <v>28</v>
       </c>
       <c r="G17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H17" s="4" t="b">
         <v>0</v>
@@ -1345,7 +1345,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
@@ -1353,22 +1353,22 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F18" t="s">
         <v>28</v>
       </c>
       <c r="G18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H18" s="4" t="b">
         <v>0</v>
@@ -1382,22 +1382,22 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E19" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F19" t="s">
         <v>28</v>
       </c>
       <c r="G19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H19" s="4" t="b">
         <v>0</v>
@@ -1406,7 +1406,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
@@ -1414,22 +1414,22 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F20" t="s">
         <v>28</v>
       </c>
       <c r="G20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H20" s="4" t="b">
         <v>0</v>
@@ -1438,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
@@ -1599,7 +1599,7 @@
         <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>
@@ -1610,7 +1610,7 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
         <v>21</v>
@@ -1621,7 +1621,7 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -1632,7 +1632,7 @@
         <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
@@ -1643,7 +1643,7 @@
         <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C7" t="s">
         <v>21</v>
@@ -1654,7 +1654,7 @@
         <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -1665,7 +1665,7 @@
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -1687,10 +1687,10 @@
         <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -1709,7 +1709,7 @@
         <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C13" t="s">
         <v>21</v>
@@ -1720,7 +1720,7 @@
         <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C14" t="s">
         <v>21</v>
@@ -1742,7 +1742,7 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C16" t="s">
         <v>21</v>
@@ -1764,10 +1764,10 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" t="s">
         <v>98</v>
-      </c>
-      <c r="C18" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -1775,7 +1775,7 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C19" t="s">
         <v>21</v>
@@ -1786,7 +1786,7 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C20" t="s">
         <v>21</v>
@@ -1800,7 +1800,7 @@
         <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -1811,7 +1811,7 @@
         <v>47</v>
       </c>
       <c r="C22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -1822,7 +1822,7 @@
         <v>48</v>
       </c>
       <c r="C23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -1919,7 +1919,7 @@
         <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1930,7 +1930,7 @@
         <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -1941,7 +1941,7 @@
         <v>59</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -1952,7 +1952,7 @@
         <v>59</v>
       </c>
       <c r="C6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1963,7 +1963,7 @@
         <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -1974,7 +1974,7 @@
         <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -1985,7 +1985,7 @@
         <v>59</v>
       </c>
       <c r="C9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -2007,7 +2007,7 @@
         <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -2029,7 +2029,7 @@
         <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -2040,7 +2040,7 @@
         <v>59</v>
       </c>
       <c r="C14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -2062,7 +2062,7 @@
         <v>59</v>
       </c>
       <c r="C16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -2084,7 +2084,7 @@
         <v>59</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -2095,7 +2095,7 @@
         <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -2106,7 +2106,7 @@
         <v>59</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -2204,7 +2204,7 @@
         <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D3" t="s">
         <v>17</v>
@@ -2218,7 +2218,7 @@
         <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
         <v>17</v>
@@ -2232,7 +2232,7 @@
         <v>59</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D5" t="s">
         <v>17</v>
@@ -2246,7 +2246,7 @@
         <v>59</v>
       </c>
       <c r="C6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D6" t="s">
         <v>17</v>
@@ -2260,7 +2260,7 @@
         <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
         <v>17</v>
@@ -2274,7 +2274,7 @@
         <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D8" t="s">
         <v>17</v>
@@ -2288,7 +2288,7 @@
         <v>59</v>
       </c>
       <c r="C9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D9" t="s">
         <v>17</v>
@@ -2316,7 +2316,7 @@
         <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D11" t="s">
         <v>17</v>
@@ -2344,7 +2344,7 @@
         <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
         <v>17</v>
@@ -2358,7 +2358,7 @@
         <v>59</v>
       </c>
       <c r="C14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D14" t="s">
         <v>17</v>
@@ -2386,7 +2386,7 @@
         <v>59</v>
       </c>
       <c r="C16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D16" t="s">
         <v>17</v>
@@ -2414,7 +2414,7 @@
         <v>59</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D18" t="s">
         <v>17</v>
@@ -2428,7 +2428,7 @@
         <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D19" t="s">
         <v>17</v>
@@ -2442,7 +2442,7 @@
         <v>59</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
         <v>17</v>

</xml_diff>